<commit_message>
Finalized notification mark seen feature
</commit_message>
<xml_diff>
--- a/student information.xlsx
+++ b/student information.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael\Documents\RESEARCH CODE (DONOTOPEN)\webportal project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B0B4628-A614-4946-84B8-512789422436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954B4C24-186E-4ACC-943F-EFFAABE24165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
   <si>
     <t>LRN</t>
   </si>
@@ -58,9 +58,6 @@
     <t>Jotham Nel Dwight R. Gamboa</t>
   </si>
   <si>
-    <t>11 CEPHEID</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nico Jade S. Abelgas </t>
   </si>
   <si>
@@ -118,13 +115,7 @@
     <t>CABANES, ROSEMARIE B.</t>
   </si>
   <si>
-    <t xml:space="preserve">James Stevin Coca </t>
-  </si>
-  <si>
     <t>11 Spica</t>
-  </si>
-  <si>
-    <t>Matt Laurence Dacayana</t>
   </si>
 </sst>
 </file>
@@ -568,10 +559,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
@@ -579,10 +570,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
@@ -590,10 +581,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -601,10 +592,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
         <v>5</v>
@@ -626,10 +617,10 @@
         <v>119874160342</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -637,10 +628,10 @@
         <v>119874131178</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -648,10 +639,10 @@
         <v>119886150058</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -659,10 +650,10 @@
         <v>119787150122</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -670,10 +661,10 @@
         <v>404491160093</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -681,10 +672,10 @@
         <v>404491160093</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -692,10 +683,10 @@
         <v>118967150018</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -703,10 +694,10 @@
         <v>119485150136</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -714,10 +705,10 @@
         <v>119880150528</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -725,10 +716,10 @@
         <v>119886150228</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -736,53 +727,30 @@
         <v>120197150018</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>119918150018</v>
-      </c>
-      <c r="B21" t="s">
-        <v>32</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="C21" s="4"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="6">
-        <v>119874150285</v>
-      </c>
-      <c r="B22" t="s">
-        <v>34</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="A22" s="6"/>
+      <c r="C22" s="4"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C23" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="C23" s="4"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C24" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="C24" s="4"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C25" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="C25" s="4"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C26" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="C26" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Refactor student list query and display formatting
</commit_message>
<xml_diff>
--- a/student information.xlsx
+++ b/student information.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael\Documents\RESEARCH CODE (DONOTOPEN)\webportal project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55422294-B061-45A3-9AF0-33A8D8A1C49F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4794C0BB-A459-43F2-8897-C62C424462A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="105">
   <si>
     <t>LRN</t>
   </si>
@@ -329,6 +329,12 @@
   </si>
   <si>
     <t>11 Mimosa</t>
+  </si>
+  <si>
+    <t>123456789444</t>
+  </si>
+  <si>
+    <t>Trying Hard</t>
   </si>
 </sst>
 </file>
@@ -463,7 +469,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -473,8 +479,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -496,7 +500,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -811,7 +815,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" style="1" customWidth="1"/>
@@ -907,840 +911,841 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="14">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="12">
         <v>119874160342</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="8">
+    <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="6">
         <v>119874131178</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B12" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="10">
-        <v>119886150058</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
+        <v>119886150058</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="6">
         <v>119787150122</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="10">
-        <v>119989160318</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
+        <v>119989160318</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="6">
         <v>404491160093</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B16" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="10">
-        <v>118967150018</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
+        <v>118967150018</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="6">
         <v>119485150136</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B18" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="10">
-        <v>119880150528</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
+        <v>119880150528</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6">
         <v>119886150228</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B20" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="10">
-        <v>120197150018</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8">
+        <v>120197150018</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="6">
         <v>119918150018</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B22" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="10">
-        <v>119874150285</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="7" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="8">
+        <v>119874150285</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="6">
         <v>119913150058</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B24" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="10">
-        <v>119893150014</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="8">
+        <v>119893150014</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="6">
         <v>119868150119</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B26" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="10">
-        <v>119793150003</v>
-      </c>
-      <c r="B26" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="8">
+        <v>119793150003</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="6">
         <v>119874160453</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B28" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C28" s="7" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="10">
-        <v>119882150204</v>
-      </c>
-      <c r="B28" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="8">
+        <v>119882150204</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="6">
         <v>119874150266</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B30" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="10">
-        <v>119886150042</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C30" s="11" t="s">
+      <c r="C30" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="8">
+        <v>119886150042</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="6">
         <v>119880150678</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B32" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="10">
-        <v>132424150032</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="7" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="8">
+        <v>132424150032</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="6">
         <v>447569150050</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B34" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C34" s="7" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="10">
-        <v>119893150570</v>
-      </c>
-      <c r="B34" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="8">
+        <v>119893150570</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="6">
         <v>1190552150001</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B36" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C36" s="7" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="10">
-        <v>119893160043</v>
-      </c>
-      <c r="B36" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="C36" s="11" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="8">
+        <v>119893160043</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="6">
         <v>119893150223</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B38" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C37" s="11" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="10">
-        <v>119145150009</v>
-      </c>
-      <c r="B38" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C38" s="11" t="s">
+      <c r="C38" s="9" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="8">
+        <v>119145150009</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="6">
         <v>119930150133</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="B40" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C39" s="9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="10">
-        <v>119918150015</v>
-      </c>
-      <c r="B40" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="8">
+        <v>119918150015</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="6">
         <v>119925150195</v>
       </c>
-      <c r="B41" s="9" t="s">
+      <c r="B42" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C42" s="7" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="10">
-        <v>119874140564</v>
-      </c>
-      <c r="B42" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="C42" s="11" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="8">
-        <v>119874150241</v>
+        <v>119874140564</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C43" s="9" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="10">
-        <v>119766160007</v>
-      </c>
-      <c r="B44" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="C44" s="11" t="s">
-        <v>96</v>
+      <c r="A44" s="6">
+        <v>119874150241</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="8">
+        <v>119766160007</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="6">
         <v>119913150226</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="B46" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C45" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="10">
-        <v>119871104277</v>
-      </c>
-      <c r="B46" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="7" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="8">
+        <v>119871104277</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="6">
         <v>119874150330</v>
       </c>
-      <c r="B47" s="9" t="s">
+      <c r="B48" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C48" s="7" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="10">
-        <v>119915150107</v>
-      </c>
-      <c r="B48" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="C48" s="11" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="8">
-        <v>119880150966</v>
+        <v>119915150107</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="10">
-        <v>120006160128</v>
-      </c>
-      <c r="B50" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C50" s="11" t="s">
+      <c r="A50" s="6">
+        <v>119880150966</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C50" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="8">
+        <v>120006160128</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="6">
         <v>119919150099</v>
       </c>
-      <c r="B51" s="9" t="s">
+      <c r="B52" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C51" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="10">
-        <v>447509150328</v>
-      </c>
-      <c r="B52" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="C52" s="11" t="s">
+      <c r="C52" s="7" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8">
+        <v>447509150328</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="6">
         <v>119873150081</v>
       </c>
-      <c r="B53" s="9" t="s">
+      <c r="B54" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C54" s="7" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="10">
-        <v>125928150010</v>
-      </c>
-      <c r="B54" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C54" s="11" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="8">
-        <v>119931150069</v>
+        <v>125928150010</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C55" s="9" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="10">
-        <v>447552150473</v>
-      </c>
-      <c r="B56" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="C56" s="11" t="s">
-        <v>97</v>
+      <c r="A56" s="6">
+        <v>119931150069</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="8">
+        <v>447552150473</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="6">
         <v>404449150097</v>
       </c>
-      <c r="B57" s="9" t="s">
+      <c r="B58" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C58" s="7" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="10">
-        <v>114750140024</v>
-      </c>
-      <c r="B58" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="C58" s="11" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="8">
+        <v>114750140024</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="6">
         <v>119886150428</v>
       </c>
-      <c r="B59" s="9" t="s">
+      <c r="B60" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C59" s="11" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="10">
-        <v>119874150810</v>
-      </c>
-      <c r="B60" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C60" s="11" t="s">
+      <c r="C60" s="9" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="8">
+        <v>119874150810</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="6">
         <v>119907150459</v>
       </c>
-      <c r="B61" s="9" t="s">
+      <c r="B62" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C61" s="11" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="10">
-        <v>119913150051</v>
-      </c>
-      <c r="B62" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C62" s="11" t="s">
+      <c r="C62" s="9" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="8">
+        <v>119913150051</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C63" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="6">
         <v>119874150569</v>
       </c>
-      <c r="B63" s="9" t="s">
+      <c r="B64" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="C63" s="11" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="10">
-        <v>119893150606</v>
-      </c>
-      <c r="B64" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="C64" s="11" t="s">
+      <c r="C64" s="9" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="8">
+        <v>119893150606</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="6">
         <v>119874150856</v>
       </c>
-      <c r="B65" s="9" t="s">
+      <c r="B66" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C65" s="11" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="10">
-        <v>119873150059</v>
-      </c>
-      <c r="B66" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="C66" s="11" t="s">
+      <c r="C66" s="9" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="8">
+        <v>119873150059</v>
+      </c>
+      <c r="B67" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="6">
         <v>447546150048</v>
       </c>
-      <c r="B67" s="9" t="s">
+      <c r="B68" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C68" s="7" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="10">
-        <v>119874160455</v>
-      </c>
-      <c r="B68" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="C68" s="11" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="8">
+        <v>119874160455</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C69" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="6">
         <v>119915150326</v>
       </c>
-      <c r="B69" s="9" t="s">
+      <c r="B70" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="C69" s="9" t="s">
+      <c r="C70" s="7" t="s">
         <v>102</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="10">
-        <v>119874150674</v>
-      </c>
-      <c r="B70" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="C70" s="11" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="8">
+        <v>119874150674</v>
+      </c>
+      <c r="B71" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C71" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="6">
         <v>119868150164</v>
       </c>
-      <c r="B71" s="9" t="s">
+      <c r="B72" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="C72" s="7" t="s">
         <v>101</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="10">
-        <v>119880150542</v>
-      </c>
-      <c r="B72" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C72" s="11" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="8">
+        <v>119880150542</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C73" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="6">
         <v>119880140706</v>
       </c>
-      <c r="B73" s="9" t="s">
+      <c r="B74" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="C73" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="10">
-        <v>119879150071</v>
-      </c>
-      <c r="B74" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="C74" s="11" t="s">
+      <c r="C74" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="8">
+        <v>119879150071</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C75" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="6">
         <v>119098150038</v>
       </c>
-      <c r="B75" s="9" t="s">
+      <c r="B76" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="C75" s="9" t="s">
+      <c r="C76" s="7" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="10">
-        <v>119871160593</v>
-      </c>
-      <c r="B76" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="C76" s="11" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="77" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="8">
+        <v>119871160593</v>
+      </c>
+      <c r="B77" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C77" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="6">
         <v>119287150034</v>
       </c>
-      <c r="B77" s="9" t="s">
+      <c r="B78" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C77" s="9" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="10">
-        <v>119893140975</v>
-      </c>
-      <c r="B78" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="C78" s="11" t="s">
+      <c r="C78" s="7" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="8">
+        <v>119893140975</v>
+      </c>
+      <c r="B79" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C79" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="6">
         <v>119874150554</v>
       </c>
-      <c r="B79" s="9" t="s">
+      <c r="B80" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="C79" s="9" t="s">
+      <c r="C80" s="7" t="s">
         <v>100</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="10">
-        <v>117205150013</v>
-      </c>
-      <c r="B80" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="C80" s="11" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="8">
+        <v>117205150013</v>
+      </c>
+      <c r="B81" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C81" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="6">
         <v>119901160299</v>
       </c>
-      <c r="B81" s="9" t="s">
+      <c r="B82" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C81" s="9" t="s">
+      <c r="C82" s="7" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="10">
+    <row r="83" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="8">
         <v>447509150275</v>
       </c>
-      <c r="B82" s="11" t="s">
+      <c r="B83" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="C82" s="11" t="s">
+      <c r="C83" s="9" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="12">
+    <row r="84" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="10">
         <v>119901150437</v>
       </c>
-      <c r="B83" s="13" t="s">
+      <c r="B84" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="C83" s="13" t="s">
+      <c r="C84" s="11" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A84" s="5"/>
-      <c r="B84" s="6"/>
-      <c r="C84" s="6"/>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A85" s="5"/>
-      <c r="B85" s="6"/>
-      <c r="C85" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Fix student login, sign-up name matching, and event/announcement deletion - Remove approval check so students on the masterlist can log in right after sign-up - Match names in any word order (Juan Cruz = Cruz, Juan) - Add ProxyFix so one student's failed logins don't lock out the whole school - Let staff delete any announcement or event - Add Posted Announcements list with Delete buttons to teacher dashboard
</commit_message>
<xml_diff>
--- a/student information.xlsx
+++ b/student information.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael\Documents\RESEARCH CODE (DONOTOPEN)\webportal project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33246DFC-7038-4C74-A916-6A8E92E1B3B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0609BE5E-0B51-446E-823F-74C7DF361236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="127">
   <si>
     <t>LRN</t>
   </si>
@@ -395,6 +395,12 @@
   </si>
   <si>
     <t xml:space="preserve">Renecycle Bilat </t>
+  </si>
+  <si>
+    <t>Butterbonia Otin</t>
+  </si>
+  <si>
+    <t>11 Wisdom</t>
   </si>
 </sst>
 </file>
@@ -773,7 +779,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" style="1" customWidth="1"/>
@@ -893,21 +899,21 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>119874160342</v>
+        <v>112233456789</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>125</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>119874131178</v>
+        <v>119874160342</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
         <v>21</v>
@@ -915,10 +921,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>119886150058</v>
+        <v>119874131178</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
         <v>21</v>
@@ -926,10 +932,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>119787150122</v>
+        <v>119886150058</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
         <v>21</v>
@@ -937,10 +943,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>119989160318</v>
+        <v>119787150122</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C15" t="s">
         <v>21</v>
@@ -948,10 +954,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>404491160093</v>
+        <v>119989160318</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C16" t="s">
         <v>21</v>
@@ -959,10 +965,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>118967150018</v>
+        <v>404491160093</v>
       </c>
       <c r="B17" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C17" t="s">
         <v>21</v>
@@ -970,10 +976,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>119485150136</v>
+        <v>118967150018</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C18" t="s">
         <v>21</v>
@@ -981,10 +987,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>119880150528</v>
+        <v>119485150136</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C19" t="s">
         <v>21</v>
@@ -992,10 +998,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>119886150228</v>
+        <v>119880150528</v>
       </c>
       <c r="B20" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
         <v>21</v>
@@ -1003,10 +1009,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>120197150018</v>
+        <v>119886150228</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C21" t="s">
         <v>21</v>
@@ -1014,21 +1020,21 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>119918150018</v>
+        <v>120197150018</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C22" t="s">
-        <v>87</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>119874150285</v>
+        <v>119918150018</v>
       </c>
       <c r="B23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C23" t="s">
         <v>87</v>
@@ -1036,21 +1042,21 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>119913150058</v>
+        <v>119874150285</v>
       </c>
       <c r="B24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C24" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>119893150014</v>
+        <v>119913150058</v>
       </c>
       <c r="B25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C25" t="s">
         <v>88</v>
@@ -1058,10 +1064,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>119868150119</v>
+        <v>119893150014</v>
       </c>
       <c r="B26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C26" t="s">
         <v>88</v>
@@ -1069,10 +1075,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>119793150003</v>
+        <v>119868150119</v>
       </c>
       <c r="B27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C27" t="s">
         <v>88</v>
@@ -1080,10 +1086,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>119874160453</v>
+        <v>119793150003</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C28" t="s">
         <v>88</v>
@@ -1091,32 +1097,32 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>119882150204</v>
+        <v>119874160453</v>
       </c>
       <c r="B29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>119874150266</v>
+        <v>119882150204</v>
       </c>
       <c r="B30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>119886150042</v>
+        <v>119874150266</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
         <v>88</v>
@@ -1124,21 +1130,21 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>119880150678</v>
+        <v>119886150042</v>
       </c>
       <c r="B32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C32" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>132424150032</v>
+        <v>119880150678</v>
       </c>
       <c r="B33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C33" t="s">
         <v>89</v>
@@ -1146,10 +1152,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>447569150050</v>
+        <v>132424150032</v>
       </c>
       <c r="B34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C34" t="s">
         <v>89</v>
@@ -1157,43 +1163,43 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>119893150570</v>
+        <v>447569150050</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C35" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>1190552150001</v>
+        <v>119893150570</v>
       </c>
       <c r="B36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C36" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>119893160043</v>
+        <v>1190552150001</v>
       </c>
       <c r="B37" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C37" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>119893150223</v>
+        <v>119893160043</v>
       </c>
       <c r="B38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
         <v>89</v>
@@ -1201,10 +1207,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>119145150009</v>
+        <v>119893150223</v>
       </c>
       <c r="B39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C39" t="s">
         <v>89</v>
@@ -1212,21 +1218,21 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>119930150133</v>
+        <v>119145150009</v>
       </c>
       <c r="B40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C40" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>119918150015</v>
+        <v>119930150133</v>
       </c>
       <c r="B41" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C41" t="s">
         <v>88</v>
@@ -1234,32 +1240,32 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>119925150195</v>
+        <v>119918150015</v>
       </c>
       <c r="B42" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C42" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>119874140564</v>
+        <v>119925150195</v>
       </c>
       <c r="B43" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C43" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>119874150241</v>
+        <v>119874140564</v>
       </c>
       <c r="B44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C44" t="s">
         <v>89</v>
@@ -1267,32 +1273,32 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>119766160007</v>
+        <v>119874150241</v>
       </c>
       <c r="B45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C45" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>119913150226</v>
+        <v>119766160007</v>
       </c>
       <c r="B46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C46" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>119871104277</v>
+        <v>119913150226</v>
       </c>
       <c r="B47" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C47" t="s">
         <v>89</v>
@@ -1300,10 +1306,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>119874150330</v>
+        <v>119871104277</v>
       </c>
       <c r="B48" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C48" t="s">
         <v>89</v>
@@ -1311,21 +1317,21 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>119915150107</v>
+        <v>119874150330</v>
       </c>
       <c r="B49" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C49" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>119880150966</v>
+        <v>119915150107</v>
       </c>
       <c r="B50" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C50" t="s">
         <v>88</v>
@@ -1333,10 +1339,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>120006160128</v>
+        <v>119880150966</v>
       </c>
       <c r="B51" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C51" t="s">
         <v>88</v>
@@ -1344,21 +1350,21 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>119919150099</v>
+        <v>120006160128</v>
       </c>
       <c r="B52" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C52" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>447509150328</v>
+        <v>119919150099</v>
       </c>
       <c r="B53" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C53" t="s">
         <v>87</v>
@@ -1366,32 +1372,32 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>119873150081</v>
+        <v>447509150328</v>
       </c>
       <c r="B54" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C54" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>125928150010</v>
+        <v>119873150081</v>
       </c>
       <c r="B55" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C55" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>119931150069</v>
+        <v>125928150010</v>
       </c>
       <c r="B56" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C56" t="s">
         <v>88</v>
@@ -1399,54 +1405,54 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>447552150473</v>
+        <v>119931150069</v>
       </c>
       <c r="B57" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C57" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>404449150097</v>
+        <v>447552150473</v>
       </c>
       <c r="B58" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C58" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>114750140024</v>
+        <v>404449150097</v>
       </c>
       <c r="B59" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C59" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>119886150428</v>
+        <v>114750140024</v>
       </c>
       <c r="B60" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C60" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>119874150810</v>
+        <v>119886150428</v>
       </c>
       <c r="B61" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C61" t="s">
         <v>93</v>
@@ -1454,10 +1460,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>119907150459</v>
+        <v>119874150810</v>
       </c>
       <c r="B62" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C62" t="s">
         <v>93</v>
@@ -1465,10 +1471,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>119913150051</v>
+        <v>119907150459</v>
       </c>
       <c r="B63" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C63" t="s">
         <v>93</v>
@@ -1476,10 +1482,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>119874150569</v>
+        <v>119913150051</v>
       </c>
       <c r="B64" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C64" t="s">
         <v>93</v>
@@ -1487,10 +1493,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>119893150606</v>
+        <v>119874150569</v>
       </c>
       <c r="B65" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C65" t="s">
         <v>93</v>
@@ -1498,10 +1504,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>119874150856</v>
+        <v>119893150606</v>
       </c>
       <c r="B66" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C66" t="s">
         <v>93</v>
@@ -1509,10 +1515,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>119873150059</v>
+        <v>119874150856</v>
       </c>
       <c r="B67" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C67" t="s">
         <v>93</v>
@@ -1520,87 +1526,87 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>447546150048</v>
+        <v>119873150059</v>
       </c>
       <c r="B68" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C68" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>119874160455</v>
+        <v>447546150048</v>
       </c>
       <c r="B69" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C69" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>119915150326</v>
+        <v>119874160455</v>
       </c>
       <c r="B70" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C70" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>119874150674</v>
+        <v>119915150326</v>
       </c>
       <c r="B71" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C71" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>119868150164</v>
+        <v>119874150674</v>
       </c>
       <c r="B72" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C72" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>119880150542</v>
+        <v>119868150164</v>
       </c>
       <c r="B73" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C73" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>119880140706</v>
+        <v>119880150542</v>
       </c>
       <c r="B74" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C74" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>119879150071</v>
+        <v>119880140706</v>
       </c>
       <c r="B75" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C75" t="s">
         <v>93</v>
@@ -1608,43 +1614,43 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>119098150038</v>
+        <v>119879150071</v>
       </c>
       <c r="B76" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C76" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>119871160593</v>
+        <v>119098150038</v>
       </c>
       <c r="B77" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C77" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>119287150034</v>
+        <v>119871160593</v>
       </c>
       <c r="B78" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="C78" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <v>119893140975</v>
+        <v>119287150034</v>
       </c>
       <c r="B79" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C79" t="s">
         <v>90</v>
@@ -1652,43 +1658,43 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <v>119874150554</v>
+        <v>119893140975</v>
       </c>
       <c r="B80" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C80" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <v>117205150013</v>
+        <v>119874150554</v>
       </c>
       <c r="B81" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C81" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <v>119901160299</v>
+        <v>117205150013</v>
       </c>
       <c r="B82" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C82" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <v>447509150275</v>
+        <v>119901160299</v>
       </c>
       <c r="B83" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C83" t="s">
         <v>91</v>
@@ -1696,65 +1702,65 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <v>119901150437</v>
+        <v>447509150275</v>
       </c>
       <c r="B84" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C84" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <v>119881150079</v>
+        <v>119901150437</v>
       </c>
       <c r="B85" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="C85" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
-        <v>119874150566</v>
+        <v>119881150079</v>
       </c>
       <c r="B86" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C86" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
-        <v>119869150058</v>
+        <v>119874150566</v>
       </c>
       <c r="B87" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C87" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <v>119880150680</v>
+        <v>119869150058</v>
       </c>
       <c r="B88" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C88" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <v>119879160105</v>
+        <v>119880150680</v>
       </c>
       <c r="B89" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C89" t="s">
         <v>91</v>
@@ -1762,10 +1768,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
-        <v>404437150046</v>
+        <v>119879160105</v>
       </c>
       <c r="B90" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C90" t="s">
         <v>91</v>
@@ -1773,10 +1779,10 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
-        <v>119881150023</v>
+        <v>404437150046</v>
       </c>
       <c r="B91" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C91" t="s">
         <v>91</v>
@@ -1784,10 +1790,10 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
-        <v>11988260181</v>
+        <v>119881150023</v>
       </c>
       <c r="B92" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C92" t="s">
         <v>91</v>
@@ -1795,10 +1801,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
-        <v>119930150021</v>
+        <v>11988260181</v>
       </c>
       <c r="B93" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C93" t="s">
         <v>91</v>
@@ -1806,10 +1812,10 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
-        <v>119893150001</v>
+        <v>119930150021</v>
       </c>
       <c r="B94" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C94" t="s">
         <v>91</v>
@@ -1817,10 +1823,10 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <v>119869150050</v>
+        <v>119893150001</v>
       </c>
       <c r="B95" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C95" t="s">
         <v>91</v>
@@ -1828,10 +1834,10 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
-        <v>119873150062</v>
+        <v>119869150050</v>
       </c>
       <c r="B96" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C96" t="s">
         <v>91</v>
@@ -1839,10 +1845,10 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
-        <v>119901150418</v>
+        <v>119873150062</v>
       </c>
       <c r="B97" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C97" t="s">
         <v>91</v>
@@ -1850,65 +1856,65 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
-        <v>119874150671</v>
+        <v>119901150418</v>
       </c>
       <c r="B98" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C98" t="s">
-        <v>123</v>
+        <v>91</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
-        <v>119874150141</v>
+        <v>119874150671</v>
       </c>
       <c r="B99" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C99" t="s">
-        <v>91</v>
+        <v>123</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
-        <v>118837150032</v>
+        <v>119874150141</v>
       </c>
       <c r="B100" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C100" t="s">
-        <v>123</v>
+        <v>91</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
-        <v>404462150148</v>
+        <v>118837150032</v>
       </c>
       <c r="B101" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C101" t="s">
-        <v>87</v>
+        <v>123</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
-        <v>404471150140</v>
+        <v>404462150148</v>
       </c>
       <c r="B102" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C102" t="s">
-        <v>123</v>
+        <v>87</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
-        <v>119919150044</v>
+        <v>404471150140</v>
       </c>
       <c r="B103" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C103" t="s">
         <v>123</v>
@@ -1916,10 +1922,10 @@
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
-        <v>120006150250</v>
+        <v>119919150044</v>
       </c>
       <c r="B104" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C104" t="s">
         <v>123</v>
@@ -1927,65 +1933,65 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
-        <v>119880160050</v>
+        <v>120006150250</v>
       </c>
       <c r="B105" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C105" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
-        <v>119868150310</v>
+        <v>119880160050</v>
       </c>
       <c r="B106" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C106" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
-        <v>119882150108</v>
+        <v>119868150310</v>
       </c>
       <c r="B107" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C107" t="s">
-        <v>123</v>
+        <v>91</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
-        <v>119263150023</v>
+        <v>119882150108</v>
       </c>
       <c r="B108" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C108" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
-        <v>119874150548</v>
+        <v>119263150023</v>
       </c>
       <c r="B109" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C109" t="s">
-        <v>123</v>
+        <v>92</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
-        <v>119868150134</v>
+        <v>119874150548</v>
       </c>
       <c r="B110" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C110" t="s">
         <v>123</v>
@@ -1993,23 +1999,34 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
-        <v>119919140079</v>
+        <v>119868150134</v>
       </c>
       <c r="B111" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C111" t="s">
-        <v>91</v>
+        <v>123</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
+        <v>119919140079</v>
+      </c>
+      <c r="B112" t="s">
+        <v>121</v>
+      </c>
+      <c r="C112" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
         <v>119881150064</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B113" t="s">
         <v>122</v>
       </c>
-      <c r="C112" t="s">
+      <c r="C113" t="s">
         <v>123</v>
       </c>
     </row>

</xml_diff>